<commit_message>
Consolidate QA scripts into unified validation format across modules
</commit_message>
<xml_diff>
--- a/nma/qa/crossval_nma_vs_r.xlsx
+++ b/nma/qa/crossval_nma_vs_r.xlsx
@@ -21,7 +21,7 @@
     <t>Published datasets: Senn 2013 (10 treatments) + Dogliotti 2014 (8 treatments)</t>
   </si>
   <si>
-    <t>Date:  7 Mar 2026</t>
+    <t>Date: 13 Mar 2026</t>
   </si>
   <si>
     <t>Dataset</t>
@@ -111,7 +111,7 @@
     <t>Summary</t>
   </si>
   <si>
-    <t>PASS: 15  NOTE: 1  FAIL: 0</t>
+    <t>PASS: 16  FAIL: 0</t>
   </si>
   <si>
     <t>Notes:</t>
@@ -1041,7 +1041,7 @@
         <v>0.88420049406435686</v>
       </c>
       <c r="E6" s="3">
-        <v>0.026000494064356894</v>
+        <v>0.026000494064356901</v>
       </c>
       <c r="F6" t="s">
         <v>11</v>
@@ -1061,7 +1061,7 @@
         <v>0.82805580560643566</v>
       </c>
       <c r="E7" s="6">
-        <v>0.088555805606435611</v>
+        <v>0.088555805606435598</v>
       </c>
       <c r="F7" t="s">
         <v>13</v>
@@ -1081,7 +1081,7 @@
         <v>1.1252883478794979</v>
       </c>
       <c r="E8" s="9">
-        <v>0.0062116521205020092</v>
+        <v>0.0062116521205019997</v>
       </c>
       <c r="F8" t="s">
         <v>11</v>
@@ -1101,7 +1101,7 @@
         <v>0.91488709339070451</v>
       </c>
       <c r="E9" s="12">
-        <v>0.035112906609295447</v>
+        <v>0.035112906609295398</v>
       </c>
       <c r="F9" t="s">
         <v>11</v>
@@ -1121,7 +1121,7 @@
         <v>1.1685810008552631</v>
       </c>
       <c r="E10" s="15">
-        <v>0.037781000855263036</v>
+        <v>0.037781000855263001</v>
       </c>
       <c r="F10" t="s">
         <v>11</v>
@@ -1141,7 +1141,7 @@
         <v>1.232537335396896</v>
       </c>
       <c r="E11" s="18">
-        <v>0.002562664603104059</v>
+        <v>0.0025626646031041002</v>
       </c>
       <c r="F11" t="s">
         <v>11</v>
@@ -1241,7 +1241,7 @@
         <v>1.107463047563126</v>
       </c>
       <c r="E16" s="33">
-        <v>0.004963047563125933</v>
+        <v>0.0049630475631259</v>
       </c>
       <c r="F16" t="s">
         <v>11</v>
@@ -1261,7 +1261,7 @@
         <v>0.28247713966582011</v>
       </c>
       <c r="E17" s="36">
-        <v>0.012077139665820136</v>
+        <v>0.012077139665820099</v>
       </c>
       <c r="F17" t="s">
         <v>11</v>
@@ -1281,7 +1281,7 @@
         <v>0.53660608819398592</v>
       </c>
       <c r="E18" s="39">
-        <v>0.013306088193985932</v>
+        <v>0.013306088193985899</v>
       </c>
       <c r="F18" t="s">
         <v>11</v>
@@ -1301,7 +1301,7 @@
         <v>0.96538038253566838</v>
       </c>
       <c r="E19" s="42">
-        <v>0.00021961746433163398</v>
+        <v>0.00021961746433159999</v>
       </c>
       <c r="F19" t="s">
         <v>11</v>
@@ -1321,7 +1321,7 @@
         <v>1.321670663010204</v>
       </c>
       <c r="E20" s="45">
-        <v>0.00022933698979610284</v>
+        <v>0.0002293369897961</v>
       </c>
       <c r="F20" t="s">
         <v>11</v>
@@ -1341,7 +1341,7 @@
         <v>1.135944298434628</v>
       </c>
       <c r="E21" s="48">
-        <v>0.00025570156537213506</v>
+        <v>0.00025570156537209999</v>
       </c>
       <c r="F21" t="s">
         <v>11</v>
@@ -1361,7 +1361,7 @@
         <v>0.88548958629320418</v>
       </c>
       <c r="E22" s="51">
-        <v>0.00021041370679586446</v>
+        <v>0.0002104137067959</v>
       </c>
       <c r="F22" t="s">
         <v>11</v>

</xml_diff>